<commit_message>
fix: improve control validation and expected price handling
Align validation waits/context to reduce false NOT FOUND outcomes.
Support expected_price_incl_vat with backward compatibility and refresh expected control data.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/expected/input_controls_expected.xlsx
+++ b/data/expected/input_controls_expected.xlsx
@@ -28,7 +28,7 @@
     <t>url</t>
   </si>
   <si>
-    <t xml:space="preserve">expected_price </t>
+    <t>expected_price_incl_vat</t>
   </si>
   <si>
     <t>expected_labels_csv</t>
@@ -43,13 +43,22 @@
     <t>https://www.justdoorsuk.com/window-order.php?product=white-window-style-1</t>
   </si>
   <si>
-    <t>Frame Width (mm), Frame Height (mm), No, 85mm Stub, Standard 150mm, 180mm, Oal Rorh Sides, Oal Rorh Sides, Anthracite Grev Both Sides, Rosewood Both Sides, Rosewood White, Anthracite Grev Both Sides, Anthracite Grev White, Chartwell White, Cream Both Sides, Cream/White, Black-Brown Both Sides, Black-Brown/White, Whitegrain Both Sides, Smooth Anthracite Grey/White, Smooth Anthracite Grey/White, Agate Grey {White, Clear, Obscure, Standard A Rated, A++ Triple Glazed, Toughened Glass, Laminated Glass, Trickle Vents, Fit Pack</t>
+    <t>Frame Width (mm), Frame Height (mm), No, 85mm Stub, Standard 150mm, 180mm, White, Oak Both Sides, Oak/White, Rosewood Both Sides, Rosewood/White, Anthracite Grev Both Sides, Anthracite Grev/White, Chartwell/White, Cream Both Sides, Cream/White, Black-Brown Both Sides, Black-Brown/White, Whitegrain Both Sides, Irish Oak Both Sides, Smooth Anthracite Grey/White, Agate Grey/White, Clear, Obscure, Standard A Rated, A+ Rated Energy Upgrade, A++ Triple Glazed, Toughened Glass, Laminated Glass, Trickle Vents, Fit Pack</t>
   </si>
   <si>
     <t>https://www.pipelagging.com/rockwool-rocklap-1m-foil-backed-pipe-insulation-lagging</t>
   </si>
   <si>
     <t>Pipe Outside Diameter mm, Insulation Thickness mm</t>
+  </si>
+  <si>
+    <t>https://www.roofingsuperstore.co.uk/product/manthorpe-gw291-intermediate-tray-rh-317mm-x-155mm.html</t>
+  </si>
+  <si>
+    <t>https://www.metals4u.co.uk/materials/stainless-steel/stainless-steel-round/1694-p</t>
+  </si>
+  <si>
+    <t>Length</t>
   </si>
 </sst>
 </file>
@@ -291,7 +300,10 @@
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="2" max="2" width="17.14063" customWidth="1"/>
+    <col min="2" max="2" width="24.85547" customWidth="1"/>
+    <col min="3" max="3" width="70.57031" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.28516" customWidth="1"/>
+    <col min="5" max="5" width="255.7109" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -316,7 +328,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2:B4" si="0">LOWER(IFERROR(IF(LEFT(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),4)="www.",MID(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),5,FIND("/",MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999)&amp;"/")-5),LEFT(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),FIND("/",MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999)&amp;"/")-1)),""))</f>
+        <f t="shared" ref="B2:B3" si="0">LOWER(IFERROR(IF(LEFT(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),4)="www.",MID(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),5,FIND("/",MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999)&amp;"/")-5),LEFT(MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999),FIND("/",MID(TRIM(C2),FIND("//",TRIM(C2)&amp;"//")+2,999)&amp;"/")-1)),""))</f>
         <v>colglo.co.uk</v>
       </c>
       <c r="C2" t="s">
@@ -352,7 +364,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" si="0"/>
+        <f>LOWER(IFERROR(IF(LEFT(MID(TRIM(C4),FIND("//",TRIM(C4)&amp;"//")+2,999),4)="www.",MID(MID(TRIM(C4),FIND("//",TRIM(C4)&amp;"//")+2,999),5,FIND("/",MID(TRIM(C4),FIND("//",TRIM(C4)&amp;"//")+2,999)&amp;"/")-5),LEFT(MID(TRIM(C4),FIND("//",TRIM(C4)&amp;"//")+2,999),FIND("/",MID(TRIM(C4),FIND("//",TRIM(C4)&amp;"//")+2,999)&amp;"/")-1)),""))</f>
         <v>pipelagging.com</v>
       </c>
       <c r="C4" t="s">
@@ -363,6 +375,39 @@
       </c>
       <c r="E4" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <f>LOWER(IFERROR(IF(LEFT(MID(TRIM(C5),FIND("//",TRIM(C5)&amp;"//")+2,999),4)="www.",MID(MID(TRIM(C5),FIND("//",TRIM(C5)&amp;"//")+2,999),5,FIND("/",MID(TRIM(C5),FIND("//",TRIM(C5)&amp;"//")+2,999)&amp;"/")-5),LEFT(MID(TRIM(C5),FIND("//",TRIM(C5)&amp;"//")+2,999),FIND("/",MID(TRIM(C5),FIND("//",TRIM(C5)&amp;"//")+2,999)&amp;"/")-1)),""))</f>
+        <v>roofingsuperstore.co.uk</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5">
+        <v>3.1200000000000001</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <f>LOWER(IFERROR(IF(LEFT(MID(TRIM(C6),FIND("//",TRIM(C6)&amp;"//")+2,999),4)="www.",MID(MID(TRIM(C6),FIND("//",TRIM(C6)&amp;"//")+2,999),5,FIND("/",MID(TRIM(C6),FIND("//",TRIM(C6)&amp;"//")+2,999)&amp;"/")-5),LEFT(MID(TRIM(C6),FIND("//",TRIM(C6)&amp;"//")+2,999),FIND("/",MID(TRIM(C6),FIND("//",TRIM(C6)&amp;"//")+2,999)&amp;"/")-1)),""))</f>
+        <v>metals4u.co.uk</v>
+      </c>
+      <c r="C6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6">
+        <v>14.34</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>